<commit_message>
AI Auditlog week 2
</commit_message>
<xml_diff>
--- a/AI_Audit_Log_TranTienDat.xlsx
+++ b/AI_Audit_Log_TranTienDat.xlsx
@@ -5,22 +5,23 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Document\Su26\SWD\AI_Auditlog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15A7F78B-D617-43C5-93B3-74A377CEA481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3B4DF2C-B62F-423A-9142-29B7743217A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="AI Audit Log TV" sheetId="1" r:id="rId1"/>
+    <sheet name="week1" sheetId="1" r:id="rId1"/>
+    <sheet name="week2" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="52">
   <si>
     <t>STT</t>
   </si>
@@ -114,6 +115,88 @@
   <si>
     <t>Phản hồi: AI cho rằng deployment modeling dùng để ánh xạ software components sang hardware environment.
 Kiểm chứng &amp; Quyết định: AI đúng nhưng chưa giải thích ảnh hưởng của distributed subsystem communication đến performance và architecture decisions. Tôi đã bổ sung mối liên hệ giữa deployment diagram, server allocation và communication overhead trong hệ thống phân tán.</t>
+  </si>
+  <si>
+    <t>“Use Case Modeling dùng để giải quyết vấn đề gì trong quá trình phát triển phần mềm?”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích Use Case Modeling giúp mô tả cách người dùng tương tác với hệ thống để xác định functional requirements.
+Kiểm chứng &amp; Quyết định: AI trả lời đúng nhưng chưa phân biệt rõ giữa yêu cầu chức năng và thiết kế hệ thống. Tôi đã bổ sung rằng Use Case chỉ tập trung vào behavior của hệ thống dưới góc nhìn người dùng chứ không mô tả cấu trúc dữ liệu hay thuật toán bên trong.</t>
+  </si>
+  <si>
+    <t>“Làm thế nào để xác định actor chính và actor phụ trong hệ thống bán hàng online?”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI cho rằng tất cả người dùng và hệ thống bên ngoài đều có thể là actor.
+Kiểm chứng &amp; Quyết định: Tôi nhận thấy AI phân loại quá rộng, dẫn đến sơ đồ bị dư actor không cần thiết. Tôi chỉ giữ lại Customer, Admin và Payment Gateway vì đây là các actor trực tiếp tương tác với hệ thống theo yêu cầu bài toán.</t>
+  </si>
+  <si>
+    <t>“Hệ thống quản lý bán hàng nên được chia thành các use case nào?”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất các use case như Login, Register, Add to Cart, Checkout và Payment.
+Kiểm chứng &amp; Quyết định: AI bỏ sót các chức năng quản trị như Manage Product và Track Order. Tôi đã bổ sung các use case cho admin để hệ thống phản ánh đầy đủ nghiệp vụ thực tế hơn.</t>
+  </si>
+  <si>
+    <t>“Làm thế nào để viết luồng sự kiện chính (Main Flow) cho Use Case Checkout?”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI mô tả quy trình checkout gồm chọn sản phẩm, nhập địa chỉ và thanh toán.
+Kiểm chứng &amp; Quyết định: Tôi nhận thấy AI chưa xử lý các trường hợp ngoại lệ như thanh toán thất bại hoặc sản phẩm hết hàng. Tôi đã bổ sung Alternative Flow và Exception Flow để mô hình use case thực tế hơn.</t>
+  </si>
+  <si>
+    <t>“Sự khác nhau giữa Include và Extend trong Use Case Diagram là gì?”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI cho rằng cả Include và Extend đều dùng để tái sử dụng chức năng giữa các use case.
+Kiểm chứng: Tôi kiểm tra lại UML Specification thì Include luôn được thực hiện bắt buộc, còn Extend chỉ xảy ra trong điều kiện đặc biệt.
+Quyết định: Tôi sử dụng Include cho “Authenticate User” và Extend cho “Apply Discount Code”. Đây là trường hợp Oversimplification của AI.</t>
+  </si>
+  <si>
+    <t>“Có cần tạo Sequence Diagram cho tất cả use case không?”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất tạo Sequence Diagram cho mọi use case để mô tả interaction đầy đủ.
+Kiểm chứng &amp; Quyết định: Tôi nhận thấy điều này không phù hợp với quy mô project nhỏ vì làm tài liệu quá lớn và khó quản lý. Tôi quyết định chỉ tạo Sequence Diagram cho các use case quan trọng như Login và Checkout để tập trung vào core functionality.</t>
+  </si>
+  <si>
+    <t>“Use Case Diagram có thể mô tả database schema và table relationships không?”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI trả lời rằng Use Case Diagram có thể dùng để mô tả dữ liệu và database relationships.
+Kiểm chứng: Tôi đối chiếu với UML documentation thì Use Case Diagram chỉ mô tả actor-system interaction chứ không mô tả database structure.
+Quyết định: Tôi loại bỏ phần database khỏi Use Case Diagram và chuyển sang ERD/Class Diagram. Đây là trường hợp Context Misunderstanding (Hallucination).</t>
+  </si>
+  <si>
+    <t>“Làm thế nào để chuyển từ Use Case Modeling sang thiết kế hệ thống MVC?”</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích rằng mỗi use case có thể được ánh xạ sang controller và service tương ứng trong kiến trúc MVC.
+Kiểm chứng &amp; Quyết định: AI trả lời đúng nhưng chưa đề cập đến việc phân chia responsibility giữa Controller, Service và DAO layer. Tôi đã bổ sung thêm tầng Service để xử lý business logic thay vì để Controller xử lý trực tiếp nhằm giảm coupling trong hệ thống.</t>
+  </si>
+  <si>
+    <t>Requirements Analysis</t>
+  </si>
+  <si>
+    <t>Actor Identification</t>
+  </si>
+  <si>
+    <t>Use Case Decomposition</t>
+  </si>
+  <si>
+    <t>Behavioral Modeling</t>
+  </si>
+  <si>
+    <t>UML Relationship Analysis</t>
+  </si>
+  <si>
+    <t>System Interaction Modeling</t>
+  </si>
+  <si>
+    <t>Verification &amp; UML Validation</t>
+  </si>
+  <si>
+    <t>Design Transition</t>
   </si>
 </sst>
 </file>
@@ -161,7 +244,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -609,4 +699,147 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0177BC5D-E419-431A-B063-84DF40B83D24}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8" style="3" customWidth="1"/>
+    <col min="2" max="2" width="30" style="3" customWidth="1"/>
+    <col min="3" max="3" width="60" style="3" customWidth="1"/>
+    <col min="4" max="4" width="100" style="3" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="120" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>